<commit_message>
Phase 2 완료 + Phase 3 설계 반영
</commit_message>
<xml_diff>
--- a/건물.xlsx
+++ b/건물.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\merge-rpg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{87037050-BFD1-4D9A-9114-A9AF4F2759D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39CE16C6-F034-483E-B849-F608223ABBD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="870" windowWidth="18225" windowHeight="14505" xr2:uid="{D81A20EF-16F9-462D-BA08-C3AF3189D473}"/>
+    <workbookView xWindow="-26280" yWindow="795" windowWidth="25290" windowHeight="14505" xr2:uid="{D81A20EF-16F9-462D-BA08-C3AF3189D473}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="51">
   <si>
     <t>농장</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -70,10 +70,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>보석</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>훈련소</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -167,6 +163,82 @@
   </si>
   <si>
     <t>효과</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>시장</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>골드</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보석(유료 재화)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>창고</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>던전 인벤토리 확장</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>지휘소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>던전 대기칸 확장</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>최대 레벨</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>건물 출현 조건 (계정 레벨)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>건물 레벨업 (출현 이후 숫자만큼 계정 레벨 업마다)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>철</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>건물 내에서 케미 효과 선택 하여 각각 레벨 업, 건물 레벨에 따라 상한</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기본 5개, 건물 레벨업 마다 인벤 +1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>건물 레벨마다 대기칸 +1 (최대 5)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>건물 레벨업 마다 효과 상승</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>비접속 시에도 재화 생산(자동 생산량은 건물 레벨마다 상한 있음 &gt; 생산 시간 제한.). 건물 레벨업 시 생산량 증가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>여신상</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스탯은 건물 레벨업 마다 상승, 캐릭터 스킬은 건물 내에서 별도로 업그레이드</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>설명</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -234,7 +306,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -243,6 +315,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -578,26 +653,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E26BEA5-14E3-411C-8411-5882B8626457}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.125" customWidth="1"/>
     <col min="2" max="2" width="21.375" customWidth="1"/>
     <col min="3" max="3" width="47.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="95.625" customWidth="1"/>
+    <col min="6" max="6" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -607,8 +697,20 @@
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="1">
+        <v>20</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -618,8 +720,20 @@
       <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="1">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1">
+        <v>3</v>
+      </c>
+      <c r="G3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -629,8 +743,20 @@
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="1">
+        <v>20</v>
+      </c>
+      <c r="F4" s="1">
+        <v>5</v>
+      </c>
+      <c r="G4" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -638,117 +764,341 @@
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="1">
+        <v>20</v>
+      </c>
+      <c r="F5" s="1">
+        <v>10</v>
+      </c>
+      <c r="G5" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="1">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1">
+        <v>15</v>
+      </c>
+      <c r="G6" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="1">
+        <v>20</v>
+      </c>
+      <c r="F7" s="1">
+        <v>5</v>
+      </c>
+      <c r="G7" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="1">
+        <v>20</v>
+      </c>
+      <c r="F8" s="1">
+        <v>10</v>
+      </c>
+      <c r="G8" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="1">
+        <v>20</v>
+      </c>
+      <c r="F9" s="1">
+        <v>10</v>
+      </c>
+      <c r="G9" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="1">
+        <v>20</v>
+      </c>
+      <c r="F10" s="1">
+        <v>15</v>
+      </c>
+      <c r="G10" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="1">
+        <v>20</v>
+      </c>
+      <c r="F11" s="1">
+        <v>15</v>
+      </c>
+      <c r="G11" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="1">
+        <v>20</v>
+      </c>
+      <c r="F12" s="1">
+        <v>20</v>
+      </c>
+      <c r="G12" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="1">
+        <v>20</v>
+      </c>
+      <c r="F13" s="1">
+        <v>20</v>
+      </c>
+      <c r="G13" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="1">
+        <v>20</v>
+      </c>
+      <c r="F14" s="1">
+        <v>20</v>
+      </c>
+      <c r="G14" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E15" s="1">
+        <v>20</v>
+      </c>
+      <c r="F15" s="1">
+        <v>20</v>
+      </c>
+      <c r="G15" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="1">
+        <v>20</v>
+      </c>
+      <c r="F16" s="1">
+        <v>20</v>
+      </c>
+      <c r="G16" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="1">
+        <v>20</v>
+      </c>
+      <c r="F17" s="1">
+        <v>25</v>
+      </c>
+      <c r="G17" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="1">
         <v>10</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
+      <c r="F18" s="1">
         <v>10</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>29</v>
+      <c r="G18" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="1">
+        <v>2</v>
+      </c>
+      <c r="F19" s="1">
+        <v>20</v>
+      </c>
+      <c r="G19" s="1">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>